<commit_message>
Før tests med filnavngivningsfejl
</commit_message>
<xml_diff>
--- a/CsvToolTests/Files/Excel/Simple data to csv.xlsx
+++ b/CsvToolTests/Files/Excel/Simple data to csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c79cbd02c8d62a0/Udvikling/Bygdrift/Tools/CsvTool/CsvToolTests/Files/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{02E0B742-73B3-4799-BBF1-F7996651DF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{607E939D-31EB-45C3-B30D-F886B2312E43}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DACD5E9B-9CA9-443C-9BCC-5DA04E750B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B5DB359A-803E-4657-A29A-BA83D94036BB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B5DB359A-803E-4657-A29A-BA83D94036BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Pane1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="11">
   <si>
     <t>Id</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>Header for pane 2</t>
+  </si>
+  <si>
+    <t>Date</t>
   </si>
 </sst>
 </file>
@@ -100,8 +103,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,15 +420,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24AB805C-FFAB-4670-A2FA-5F28BD585B28}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -432,61 +436,79 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>7.2</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1">
+        <v>45658</v>
+      </c>
+      <c r="D4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1">
+        <v>45905</v>
+      </c>
+      <c r="D5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
       <c r="B6">
         <v>8</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1">
+        <v>45906</v>
+      </c>
+      <c r="D6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>4</v>
       </c>
       <c r="B7">
         <v>4</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1">
+        <v>45907</v>
+      </c>
+      <c r="D7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
       <c r="B8">
         <v>6.2</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1">
+        <v>45908</v>
+      </c>
+      <c r="D8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -498,14 +520,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D77D6D3-312A-4D6C-94C8-62EB1CCFE745}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -516,7 +538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>1</v>
       </c>
@@ -527,7 +549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>2</v>
       </c>
@@ -538,7 +560,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>3</v>
       </c>
@@ -549,7 +571,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>4</v>
       </c>
@@ -560,7 +582,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>5</v>
       </c>

</xml_diff>